<commit_message>
test: record final zero-operation and parameterized export acceptance
</commit_message>
<xml_diff>
--- a/docs/qa/protocol-consistency-20261007/evidence/experiment.xlsx
+++ b/docs/qa/protocol-consistency-20261007/evidence/experiment.xlsx
@@ -76,13 +76,13 @@
     <t>tags</t>
   </si>
   <si>
-    <t>测试执行一致性 1791355538054</t>
-  </si>
-  <si>
-    <t>RPL-QA-1791355538054</t>
-  </si>
-  <si>
-    <t>EXP-069</t>
+    <t>测试执行一致性 1791355947542</t>
+  </si>
+  <si>
+    <t>RPL-QA-1791355947542</t>
+  </si>
+  <si>
+    <t>EXP-088</t>
   </si>
   <si>
     <t>测试浏览器实际创建</t>
@@ -97,7 +97,7 @@
     <t>draft</t>
   </si>
   <si>
-    <t>PRT-938054</t>
+    <t>PRT-947542</t>
   </si>
   <si>
     <t>1.0</t>
@@ -119,7 +119,7 @@
 合成示例
 200 µL
 参考资料：结构验证使用合成内容，不构成实验建议。
-PRT-938054 · 合成多段步骤验收 · v1.0
+PRT-947542 · 合成多段步骤验收 · v1.0
 ✓ 准备示例 A
 偏差：测试备注必须保存
 完整说明 200 µL，20–25°C；观察标记。
@@ -137,7 +137,7 @@
 重复洗涤操作需要单独保留；实际体积 40 µL。</t>
   </si>
   <si>
-    <t>[2026-10-07T06:45:49.990Z]
+    <t>[2026-10-07T06:52:39.425Z]
 Run parameters changed: {} → {"dose":"19"}</t>
   </si>
 </sst>

</xml_diff>